<commit_message>
chore: checkpoint current workspace changes
</commit_message>
<xml_diff>
--- a/tmp/IDE问题清单.xlsx
+++ b/tmp/IDE问题清单.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joii\project\cpq\tmp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C31AD55-4895-439F-A85A-77CC1A6B61C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE5AB3EA-8DF9-430E-8EA1-84AE8CFB8C71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="28395" windowHeight="14640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="405" yWindow="840" windowWidth="28395" windowHeight="14640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>验证中</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -631,6 +631,50 @@
   <si>
     <t>IDE中,不同的容器中的AI对 "部署" 的命令行为不一致, 有的是部署到Appsmith,有的是同步的git. 
 要求: 相同的命令"部署"让AI的行为达到一致的效果</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>这是没有触发了删除的, createdAt是6月23日 正常的日期
+    "unpublishedAction": {
+        "name": "check_action",
+        "fullyQualifiedName": "VALID.check_action",
+        "datasource": {
+            "name": "UNUSED_DATASOURCE",
+            "pluginId": "64a257324cec4f198aa05848",
+            "workspaceId": "64a3df72eca3553cdfdc423c",
+            "createdAt": ISODate("2026-06-23T08:50:15.97Z"),
+            "updatedAt": ISODate("2026-09-28T08:13:02.597Z"),
+            "deleted": false,
+            "policies": [ ]
+        },
+这是触发了删除的,createdAt:是最新的日期
+    "unpublishedAction": {
+        "name": "insert",
+        "fullyQualifiedName": "PROCESS.insert",
+        "datasource": {
+            "name": "UNUSED_DATASOURCE",
+            "pluginId": "64a257324cec4f198aa05848",
+            "workspaceId": "64a3df72eca3553cdfdc423c",
+            "createdAt": ISODate("2026-09-28T07:11:35.413Z"),
+            "updatedAt": ISODate("2026-09-28T08:09:02.222Z"),
+            "deleted": false,
+            "policies": [ ]
+        },</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>执行部署后,会存在将newAction表中的数据删除
+并且删除后没有恢复插入,执行部署后,整个PROCESS的js文件丢失</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">IDE中使用CODEX提问时,会自动读取skill并修改代码.
+使用时提出的问题可能与项目无关,也会走这套流程去执行.
+</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>要有一个开关,关闭后所有提问与项目无关,不需要加载skill,只需要回答问题即可</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -772,19 +816,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -798,6 +836,15 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -807,13 +854,13 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1110,16 +1157,16 @@
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="2"/>
@@ -1135,34 +1182,34 @@
       <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
-      <c r="J2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
+      <c r="J2" s="12"/>
       <c r="K2" s="2"/>
     </row>
     <row r="3" spans="1:11" ht="75.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="13"/>
       <c r="K3" s="2" t="s">
         <v>9</v>
       </c>
@@ -1171,34 +1218,34 @@
       <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="12"/>
-      <c r="H4" s="12"/>
-      <c r="I4" s="12"/>
-      <c r="J4" s="12"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="14"/>
       <c r="K4" s="2"/>
     </row>
     <row r="5" spans="1:11" ht="90.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
       <c r="K5" s="2" t="s">
         <v>11</v>
       </c>
@@ -1207,17 +1254,17 @@
       <c r="A6" s="2">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
       <c r="K6" s="2" t="s">
         <v>10</v>
       </c>
@@ -1226,17 +1273,17 @@
       <c r="A7" s="2">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
+      <c r="I7" s="15"/>
+      <c r="J7" s="15"/>
       <c r="K7" s="2" t="s">
         <v>15</v>
       </c>
@@ -1245,119 +1292,127 @@
       <c r="A8" s="2">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
       <c r="K8" s="2"/>
     </row>
-    <row r="9" spans="1:11" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" ht="163.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>8</v>
       </c>
-      <c r="B9" s="13"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="13"/>
-      <c r="J9" s="13"/>
-      <c r="K9" s="2"/>
+      <c r="B9" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
+      <c r="J9" s="15"/>
+      <c r="K9" s="7" t="s">
+        <v>17</v>
+      </c>
     </row>
-    <row r="10" spans="1:11" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" ht="74.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
         <v>9</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
-      <c r="H10" s="13"/>
-      <c r="I10" s="13"/>
-      <c r="J10" s="13"/>
-      <c r="K10" s="2"/>
+      <c r="B10" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15"/>
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="2" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="11" spans="1:11" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
         <v>10</v>
       </c>
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="13"/>
-      <c r="J11" s="13"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
       <c r="K11" s="2"/>
     </row>
     <row r="12" spans="1:11" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
         <v>11</v>
       </c>
-      <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="13"/>
-      <c r="J12" s="13"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
       <c r="K12" s="2"/>
     </row>
     <row r="13" spans="1:11" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
         <v>12</v>
       </c>
-      <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
-      <c r="H13" s="13"/>
-      <c r="I13" s="13"/>
-      <c r="J13" s="13"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
       <c r="K13" s="2"/>
     </row>
     <row r="14" spans="1:11" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
         <v>13</v>
       </c>
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-      <c r="H14" s="13"/>
-      <c r="I14" s="13"/>
-      <c r="J14" s="13"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
       <c r="K14" s="2"/>
     </row>
     <row r="15" spans="1:11" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="14">

</xml_diff>